<commit_message>
Isolate DZL Auto-Replenishment plan and export separate Excel files
</commit_message>
<xml_diff>
--- a/Reports/TY Sep_Target.xlsx
+++ b/Reports/TY Sep_Target.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="14856" windowHeight="10968"/>
+    <workbookView windowWidth="23040" windowHeight="10440"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>Profit Center / Cost Center</t>
   </si>
@@ -114,18 +114,109 @@
   </si>
   <si>
     <t>Total</t>
+  </si>
+  <si>
+    <r>
+      <t>K104</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: DZL Uwalk Riyadh</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>K107</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: DZL Riyadh Park</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>K111</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: DZL Solitaire</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>K206</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> DZL Uwalk Jeddah</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>K204</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> DZL Redsea</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>K502</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> DZL Tabuk</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="42" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="176" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="177" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="23">
     <font>
@@ -827,7 +918,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -862,6 +953,7 @@
     <xf numFmtId="49" fontId="1" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1181,10 +1273,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="24.3333333333333" customWidth="1"/>
+    <col min="2" max="2" width="11.7777777777778"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1351,7 +1444,7 @@
         <v>180310</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" ht="22.8" spans="1:2">
       <c r="A23" s="9" t="s">
         <v>23</v>
       </c>
@@ -1394,6 +1487,54 @@
     <row r="28" spans="1:2">
       <c r="A28" s="11" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30" s="12">
+        <v>68372</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31" s="12">
+        <v>226972</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32" s="12">
+        <v>204400</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33" s="12">
+        <v>58433</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34" s="12">
+        <v>173185</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35" s="12">
+        <v>40426</v>
       </c>
     </row>
   </sheetData>

</xml_diff>